<commit_message>
adding zombies_marginals.xlsx and zombies_marginals_without_cortana.xlsx
</commit_message>
<xml_diff>
--- a/social_data/zombies_social_data/zombies_marginals.xlsx
+++ b/social_data/zombies_social_data/zombies_marginals.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t xml:space="preserve">MonkeyName</t>
   </si>
@@ -59,6 +59,18 @@
   </si>
   <si>
     <t xml:space="preserve">AffiliationFrom81G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Family</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sex</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rank</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grouping</t>
   </si>
   <si>
     <t xml:space="preserve">69X</t>
@@ -100,6 +112,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -186,14 +199,14 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:R11"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18.47"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14.72"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="15.84"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="18.06"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="15.69"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="15.68"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="18.06"/>
   </cols>
   <sheetData>
@@ -237,6 +250,18 @@
       <c r="M1" s="0" t="s">
         <v>12</v>
       </c>
+      <c r="N1" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="0" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="n">
@@ -278,15 +303,23 @@
       <c r="M2" s="1" t="n">
         <v>17</v>
       </c>
-      <c r="N2" s="1"/>
-      <c r="O2" s="1"/>
-      <c r="P2" s="1"/>
-      <c r="Q2" s="1"/>
+      <c r="N2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="O2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="P2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q2" s="1" t="n">
+        <v>3</v>
+      </c>
       <c r="R2" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B3" s="0" t="n">
         <v>184</v>
@@ -324,10 +357,22 @@
       <c r="M3" s="0" t="n">
         <v>18</v>
       </c>
+      <c r="N3" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="O3" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q3" s="0" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B4" s="0" t="n">
         <v>144</v>
@@ -365,10 +410,22 @@
       <c r="M4" s="0" t="n">
         <v>43</v>
       </c>
+      <c r="N4" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="O4" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q4" s="0" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="B5" s="0" t="n">
         <v>219</v>
@@ -406,10 +463,22 @@
       <c r="M5" s="0" t="n">
         <v>34</v>
       </c>
+      <c r="N5" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="O5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q5" s="0" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B6" s="0" t="n">
         <v>167</v>
@@ -447,10 +516,22 @@
       <c r="M6" s="0" t="n">
         <v>10</v>
       </c>
+      <c r="N6" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="O6" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q6" s="0" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B7" s="0" t="n">
         <v>128</v>
@@ -488,10 +569,22 @@
       <c r="M7" s="0" t="n">
         <v>23</v>
       </c>
+      <c r="N7" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="O7" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q7" s="0" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B8" s="0" t="n">
         <v>190</v>
@@ -529,10 +622,22 @@
       <c r="M8" s="0" t="n">
         <v>0</v>
       </c>
+      <c r="N8" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q8" s="0" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B9" s="0" t="n">
         <v>182</v>
@@ -570,10 +675,22 @@
       <c r="M9" s="0" t="n">
         <v>34</v>
       </c>
+      <c r="N9" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="O9" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q9" s="0" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="B10" s="0" t="n">
         <v>62</v>
@@ -611,10 +728,22 @@
       <c r="M10" s="0" t="n">
         <v>2</v>
       </c>
+      <c r="N10" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="O10" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="P10" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q10" s="0" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B11" s="0" t="n">
         <v>53</v>
@@ -651,6 +780,18 @@
       </c>
       <c r="M11" s="0" t="n">
         <v>9</v>
+      </c>
+      <c r="N11" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="O11" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="P11" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q11" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>